<commit_message>
Ajustes generación reporte endoso
</commit_message>
<xml_diff>
--- a/Documentación/brecha fianzas.xlsx
+++ b/Documentación/brecha fianzas.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0569547D-3AD1-4703-8243-92CE68B0F26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74033CA6-BCAF-4C45-9C3D-FAE8283028CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Fianza - Emision" sheetId="3" r:id="rId1"/>
-    <sheet name="Fianza - Reaseguro" sheetId="4" r:id="rId2"/>
-    <sheet name="Fianza - Contacto" sheetId="5" r:id="rId3"/>
-    <sheet name="EjemploCumulo" sheetId="2" r:id="rId4"/>
-    <sheet name="Notas" sheetId="1" r:id="rId5"/>
+    <sheet name="Fianza-Endoso" sheetId="6" r:id="rId2"/>
+    <sheet name="Fianza - Reaseguro" sheetId="4" r:id="rId3"/>
+    <sheet name="Fianza - Contacto" sheetId="5" r:id="rId4"/>
+    <sheet name="EjemploCumulo" sheetId="2" r:id="rId5"/>
+    <sheet name="Notas" sheetId="1" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="181">
   <si>
     <t>Agregar opción de gestión de coberturas</t>
   </si>
@@ -301,9 +302,6 @@
 3. Ver en versión de GLOBAL manejo de Gasto por parte de coaseguro cuando se perfila como un participante y no lider</t>
   </si>
   <si>
-    <t>Validar</t>
-  </si>
-  <si>
     <t>1. Actualmente el sistema cuenta con los cálculos de cúmulo por cliente, póliza y GEC, sin embargo, no cuenta con la validación correcta para consorcios.
 2. Se debe validar que para un consorcio el sistema ejecute un cúmulo por cada empresa o contacto incluido en el grupo económico y si uno de esta empresas tiene GEC debe evaluarse correctamente.</t>
   </si>
@@ -487,6 +485,133 @@
   </si>
   <si>
     <t>Desarrollar y configurar en todos los productos de fianzas</t>
+  </si>
+  <si>
+    <t>Cúmulo Detalle</t>
+  </si>
+  <si>
+    <t>Endosos</t>
+  </si>
+  <si>
+    <t>Formato endoso</t>
+  </si>
+  <si>
+    <t>Habilitar formato de endoso según GLOBAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambio de vigencia, mueve las fechas de las coberturas, validando ls coberturas dependientes, no afecta ni prima ni suma, solo vigencias
+No Afecta reaseguro
+Actualiza la vigencia de la fianza
+Si no se marca la opción de orden de proceder no se debe permitir ejecutar el endoso de orden de proceder
+En fianza garantia cumplimiento de gobierno se debe marcar automáticamente la orden de proceder
+En facturación histórica se deben ver todos los movimientos
+</t>
+  </si>
+  <si>
+    <t>Extensión de vigencia</t>
+  </si>
+  <si>
+    <t>Se pueden mover cobertura principal y cobertura de mantenimiento
+Se puede mover fecha final de la cobertura de mantenimiento
+Endoso permite aplicar un descuento/recargo inmerso en el mismo endoso de extensión
+Genera su respectivo reaseguro
+Poder modificar el reaseguro antes de confirmar
+SE mueven las fechas de las coberturas en base a la configuración de principal-dependientes
+Ver cómo lo hace sis9 para calcular la extensión/reducción de vigencia</t>
+  </si>
+  <si>
+    <t>Se genera reaseguro previo a confirmar y modificarlo antes de confirmar.</t>
+  </si>
+  <si>
+    <t>Bordereau</t>
+  </si>
+  <si>
+    <t>Se puede modificar el número del endoso posterior a confirmarlo</t>
+  </si>
+  <si>
+    <t>Cancelación</t>
+  </si>
+  <si>
+    <t>Sis9 cancela cada recibo por separado</t>
+  </si>
+  <si>
+    <t>Estado Fianza</t>
+  </si>
+  <si>
+    <t>Validar que todo movimientos se refleje correctamente en el borderó
+Validar diseño de bordereau de emisión vs sis9, ver filtros y diseño</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver si podemos definir una vigencia automática </t>
+  </si>
+  <si>
+    <t>Validar si el sistema cotiza o simplementa aplica prorrata</t>
+  </si>
+  <si>
+    <t>Cambio de SA</t>
+  </si>
+  <si>
+    <t>Endoso de cambio de OA</t>
+  </si>
+  <si>
+    <t>Jessica enviará lista para campos editables
+Modificar Garantías (valor - descripción)</t>
+  </si>
+  <si>
+    <t>Cuotas</t>
+  </si>
+  <si>
+    <t>Validar con Linneth el calendario de pagos de fianzas</t>
+  </si>
+  <si>
+    <t>Cambio de forma de pago</t>
+  </si>
+  <si>
+    <t>Validar consecutivo de endoso, debería ser 1 para identificar que es interno</t>
+  </si>
+  <si>
+    <t>Mapa del ente</t>
+  </si>
+  <si>
+    <t>Ver mapa del ente, validar cómo funciona en sis11</t>
+  </si>
+  <si>
+    <t>Renovación</t>
+  </si>
+  <si>
+    <t>Fianzas judiciales se renuevan y fianzas miscelaneas ramo 83 y 84</t>
+  </si>
+  <si>
+    <t>Endoso de Orden de proceder</t>
+  </si>
+  <si>
+    <t>Endoso</t>
+  </si>
+  <si>
+    <t>Validar y Ajustar</t>
+  </si>
+  <si>
+    <t>Emision</t>
+  </si>
+  <si>
+    <t>Existe un estado de activo o inactivo, por ahora no se atenderá, se validará la necesidad previamente</t>
+  </si>
+  <si>
+    <t>Validar y Configurar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El contrato no tiene configuración definida en facultativo de reaseguradores, se solicita con cada caso
+Se valida la distribución de reaseguradores
+Montar reaseguradores y corredores (Catalogo)
+Habilitar corredor en el formulario de reaseguro </t>
+  </si>
+  <si>
+    <t>Esperar</t>
+  </si>
+  <si>
+    <t>Se requiere una vista en dónde se pueda consultar el cúmulo de fianzas vigentes por cliente, póliza y grupo económico
+Cumulo solo para fianzas
+Solo fianzas vigentes - No canceladas y según vigencia</t>
   </si>
 </sst>
 </file>
@@ -541,7 +666,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -559,12 +684,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -884,7 +1017,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" style="8" bestFit="1" customWidth="1"/>
@@ -894,8 +1027,7 @@
     <col min="5" max="5" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7" style="8" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="108.7109375" style="11" customWidth="1"/>
-    <col min="9" max="16384" width="11.42578125" style="9"/>
+    <col min="8" max="8" width="108.7109375" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -920,7 +1052,7 @@
       <c r="G1" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>57</v>
       </c>
     </row>
@@ -946,7 +1078,7 @@
       <c r="G2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="9" t="s">
         <v>74</v>
       </c>
     </row>
@@ -972,7 +1104,7 @@
       <c r="G3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="9" t="s">
         <v>77</v>
       </c>
     </row>
@@ -998,68 +1130,68 @@
       <c r="G4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="B6" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>61</v>
-      </c>
       <c r="G6" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>88</v>
+        <v>134</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>58</v>
@@ -1071,13 +1203,13 @@
         <v>60</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H7" s="10" t="s">
-        <v>145</v>
+      <c r="H7" s="9" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1085,31 +1217,33 @@
         <v>8</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>58</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="H8" s="10"/>
+        <v>62</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>58</v>
@@ -1126,8 +1260,8 @@
       <c r="G9" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H9" s="10" t="s">
-        <v>90</v>
+      <c r="H9" s="9" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1135,51 +1269,49 @@
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>58</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>91</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="H10" s="9"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>89</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1187,7 +1319,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>58</v>
@@ -1204,16 +1336,16 @@
       <c r="G12" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H12" s="10" t="s">
-        <v>93</v>
+      <c r="H12" s="9" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>89</v>
+      <c r="B13" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>58</v>
@@ -1230,16 +1362,16 @@
       <c r="G13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H13" s="11" t="s">
-        <v>94</v>
+      <c r="H13" s="9" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>89</v>
+      <c r="B14" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>58</v>
@@ -1256,8 +1388,8 @@
       <c r="G14" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H14" s="11" t="s">
-        <v>95</v>
+      <c r="H14" s="9" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1265,7 +1397,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>58</v>
@@ -1282,8 +1414,8 @@
       <c r="G15" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H15" s="11" t="s">
-        <v>96</v>
+      <c r="H15" s="10" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1291,7 +1423,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>58</v>
@@ -1308,8 +1440,8 @@
       <c r="G16" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H16" s="11" t="s">
-        <v>97</v>
+      <c r="H16" s="10" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1317,7 +1449,7 @@
         <v>8</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>58</v>
@@ -1334,8 +1466,8 @@
       <c r="G17" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H17" s="11" t="s">
-        <v>98</v>
+      <c r="H17" s="10" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1343,7 +1475,7 @@
         <v>8</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>58</v>
@@ -1360,8 +1492,8 @@
       <c r="G18" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H18" s="11" t="s">
-        <v>99</v>
+      <c r="H18" s="10" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1369,7 +1501,7 @@
         <v>8</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>58</v>
@@ -1386,8 +1518,8 @@
       <c r="G19" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H19" s="11" t="s">
-        <v>100</v>
+      <c r="H19" s="10" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1395,7 +1527,7 @@
         <v>8</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>58</v>
@@ -1412,8 +1544,8 @@
       <c r="G20" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H20" s="11" t="s">
-        <v>101</v>
+      <c r="H20" s="10" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1421,7 +1553,7 @@
         <v>8</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>58</v>
@@ -1438,8 +1570,8 @@
       <c r="G21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H21" s="11" t="s">
-        <v>102</v>
+      <c r="H21" s="10" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1447,7 +1579,7 @@
         <v>8</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>58</v>
@@ -1464,8 +1596,8 @@
       <c r="G22" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H22" s="11" t="s">
-        <v>103</v>
+      <c r="H22" s="10" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1473,7 +1605,7 @@
         <v>8</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>58</v>
@@ -1490,8 +1622,8 @@
       <c r="G23" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H23" s="11" t="s">
-        <v>104</v>
+      <c r="H23" s="10" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1499,7 +1631,7 @@
         <v>8</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>58</v>
@@ -1516,8 +1648,8 @@
       <c r="G24" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H24" s="11" t="s">
-        <v>105</v>
+      <c r="H24" s="10" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1525,7 +1657,7 @@
         <v>8</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>58</v>
@@ -1542,8 +1674,8 @@
       <c r="G25" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H25" s="11" t="s">
-        <v>106</v>
+      <c r="H25" s="10" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1551,7 +1683,7 @@
         <v>8</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>58</v>
@@ -1568,8 +1700,8 @@
       <c r="G26" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H26" s="11" t="s">
-        <v>107</v>
+      <c r="H26" s="10" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -1577,7 +1709,7 @@
         <v>8</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>58</v>
@@ -1594,8 +1726,8 @@
       <c r="G27" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H27" s="11" t="s">
-        <v>108</v>
+      <c r="H27" s="10" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1603,7 +1735,7 @@
         <v>8</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>58</v>
@@ -1620,8 +1752,8 @@
       <c r="G28" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H28" s="11" t="s">
-        <v>109</v>
+      <c r="H28" s="10" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1629,7 +1761,7 @@
         <v>8</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>58</v>
@@ -1646,8 +1778,8 @@
       <c r="G29" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H29" s="11" t="s">
-        <v>110</v>
+      <c r="H29" s="10" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1655,7 +1787,7 @@
         <v>8</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>58</v>
@@ -1672,8 +1804,8 @@
       <c r="G30" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H30" s="11" t="s">
-        <v>111</v>
+      <c r="H30" s="10" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -1681,7 +1813,7 @@
         <v>8</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>58</v>
@@ -1698,8 +1830,8 @@
       <c r="G31" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H31" s="11" t="s">
-        <v>112</v>
+      <c r="H31" s="10" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1707,7 +1839,7 @@
         <v>8</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>58</v>
@@ -1724,8 +1856,8 @@
       <c r="G32" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H32" s="11" t="s">
-        <v>113</v>
+      <c r="H32" s="10" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
@@ -1733,7 +1865,7 @@
         <v>8</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>58</v>
@@ -1750,8 +1882,8 @@
       <c r="G33" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H33" s="11" t="s">
-        <v>114</v>
+      <c r="H33" s="10" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1759,7 +1891,7 @@
         <v>8</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>58</v>
@@ -1776,8 +1908,8 @@
       <c r="G34" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H34" s="11" t="s">
-        <v>115</v>
+      <c r="H34" s="10" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -1785,7 +1917,7 @@
         <v>8</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>58</v>
@@ -1802,8 +1934,8 @@
       <c r="G35" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H35" s="11" t="s">
-        <v>116</v>
+      <c r="H35" s="10" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -1811,7 +1943,7 @@
         <v>8</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>58</v>
@@ -1828,8 +1960,8 @@
       <c r="G36" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H36" s="11" t="s">
-        <v>117</v>
+      <c r="H36" s="10" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -1837,7 +1969,7 @@
         <v>8</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>58</v>
@@ -1854,8 +1986,8 @@
       <c r="G37" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H37" s="11" t="s">
-        <v>118</v>
+      <c r="H37" s="10" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -1863,7 +1995,7 @@
         <v>8</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>58</v>
@@ -1880,8 +2012,8 @@
       <c r="G38" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H38" s="11" t="s">
-        <v>119</v>
+      <c r="H38" s="10" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -1889,7 +2021,7 @@
         <v>8</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>58</v>
@@ -1906,8 +2038,8 @@
       <c r="G39" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H39" s="11" t="s">
-        <v>120</v>
+      <c r="H39" s="10" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -1915,7 +2047,7 @@
         <v>8</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>58</v>
@@ -1932,8 +2064,8 @@
       <c r="G40" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H40" s="11" t="s">
-        <v>121</v>
+      <c r="H40" s="10" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -1941,7 +2073,7 @@
         <v>8</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>58</v>
@@ -1958,8 +2090,8 @@
       <c r="G41" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H41" s="11" t="s">
-        <v>122</v>
+      <c r="H41" s="10" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1967,7 +2099,7 @@
         <v>8</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>58</v>
@@ -1984,8 +2116,8 @@
       <c r="G42" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H42" s="11" t="s">
-        <v>123</v>
+      <c r="H42" s="10" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1993,7 +2125,7 @@
         <v>8</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>58</v>
@@ -2010,8 +2142,8 @@
       <c r="G43" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H43" s="11" t="s">
-        <v>124</v>
+      <c r="H43" s="10" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2019,7 +2151,7 @@
         <v>8</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>58</v>
@@ -2036,8 +2168,8 @@
       <c r="G44" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H44" s="11" t="s">
-        <v>125</v>
+      <c r="H44" s="10" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2045,7 +2177,7 @@
         <v>8</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>58</v>
@@ -2062,8 +2194,8 @@
       <c r="G45" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H45" s="11" t="s">
-        <v>126</v>
+      <c r="H45" s="10" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2071,7 +2203,7 @@
         <v>8</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>58</v>
@@ -2088,8 +2220,8 @@
       <c r="G46" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H46" s="11" t="s">
-        <v>127</v>
+      <c r="H46" s="10" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2097,7 +2229,7 @@
         <v>8</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>58</v>
@@ -2114,8 +2246,8 @@
       <c r="G47" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H47" s="11" t="s">
-        <v>128</v>
+      <c r="H47" s="10" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2123,7 +2255,7 @@
         <v>8</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>58</v>
@@ -2140,8 +2272,8 @@
       <c r="G48" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H48" s="11" t="s">
-        <v>129</v>
+      <c r="H48" s="10" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -2149,7 +2281,7 @@
         <v>8</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>58</v>
@@ -2166,8 +2298,8 @@
       <c r="G49" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H49" s="11" t="s">
-        <v>130</v>
+      <c r="H49" s="10" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2175,7 +2307,7 @@
         <v>8</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>58</v>
@@ -2192,8 +2324,8 @@
       <c r="G50" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H50" s="11" t="s">
-        <v>131</v>
+      <c r="H50" s="10" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2201,7 +2333,7 @@
         <v>8</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>58</v>
@@ -2218,8 +2350,8 @@
       <c r="G51" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H51" s="11" t="s">
-        <v>132</v>
+      <c r="H51" s="10" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2227,7 +2359,7 @@
         <v>8</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>58</v>
@@ -2244,8 +2376,8 @@
       <c r="G52" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H52" s="11" t="s">
-        <v>133</v>
+      <c r="H52" s="10" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -2253,7 +2385,7 @@
         <v>8</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>58</v>
@@ -2270,8 +2402,86 @@
       <c r="G53" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H53" s="11" t="s">
-        <v>134</v>
+      <c r="H53" s="10" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H54" s="10" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H55" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="H56" s="11" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2280,18 +2490,351 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB8B47E-08E9-4DD4-A45C-9428CAA77C43}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" style="13"/>
+    <col min="8" max="8" width="121" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D9EB435-5367-49EB-A688-24EC17C83E2C}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A2:H5"/>
+  <dimension ref="A2:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="11.42578125" style="8"/>
     <col min="7" max="7" width="13.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="120.5703125" style="11" customWidth="1"/>
+    <col min="8" max="8" width="120.5703125" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2316,7 +2859,7 @@
       <c r="G2" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="9" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2342,7 +2885,7 @@
       <c r="G3" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="9" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2368,7 +2911,7 @@
       <c r="G4" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="H4" s="11" t="s">
+      <c r="H4" s="10" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2383,19 +2926,71 @@
         <v>58</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>72</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>86</v>
+    </row>
+    <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2403,12 +2998,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49E5BA13-0CF1-4844-871E-AC162DBE5D4C}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16.7109375" style="8" bestFit="1" customWidth="1"/>
@@ -2421,7 +3016,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D1" s="8"/>
-      <c r="H1" s="11"/>
+      <c r="H1" s="10"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
@@ -2445,16 +3040,16 @@
       <c r="G2" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="9" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>58</v>
@@ -2469,18 +3064,18 @@
         <v>72</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>142</v>
+        <v>137</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>58</v>
@@ -2498,12 +3093,12 @@
         <v>62</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>32</v>
@@ -2524,12 +3119,12 @@
         <v>62</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>41</v>
@@ -2547,10 +3142,36 @@
         <v>72</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2558,7 +3179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E1CF682-82A7-4821-BF8C-AA66C43E8BCE}">
   <dimension ref="A2:I33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2831,7 +3452,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF353B9A-6E8D-46D8-B856-D5F5A0A602CB}">
   <dimension ref="B2:M22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>